<commit_message>
legacy imaging v9: archive old seed kits, add v2 pipeline, and update constructs/tags
</commit_message>
<xml_diff>
--- a/seed_kits/2025-11-15-121231-autoload/tags.xlsx
+++ b/seed_kits/2025-11-15-121231-autoload/tags.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/davekokel/Projects/carp_v2/seed_kits/2025-11-15-121231-autoload/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A281C69A-3512-9A44-BFCB-CE2AA6739B6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C148F9E-36CA-0A4B-B02E-D16F074DACE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32960" yWindow="16860" windowWidth="27640" windowHeight="16680" xr2:uid="{89706445-C364-CF42-9B42-6F31A2F723ED}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34560" windowHeight="19860" xr2:uid="{89706445-C364-CF42-9B42-6F31A2F723ED}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$A$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$A$44</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="42">
   <si>
     <t>2Xcox8A</t>
   </si>
@@ -120,6 +120,51 @@
   </si>
   <si>
     <t>aliases</t>
+  </si>
+  <si>
+    <t>skl</t>
+  </si>
+  <si>
+    <t>Peroxisome</t>
+  </si>
+  <si>
+    <t>EB3</t>
+  </si>
+  <si>
+    <t>Microtubule EBP</t>
+  </si>
+  <si>
+    <t>cortactin</t>
+  </si>
+  <si>
+    <t>Lamellipodia</t>
+  </si>
+  <si>
+    <t>ABCDpmp70</t>
+  </si>
+  <si>
+    <t>calnexin</t>
+  </si>
+  <si>
+    <t>LEMD2</t>
+  </si>
+  <si>
+    <t>Nuclear Envelope</t>
+  </si>
+  <si>
+    <t>pex3</t>
+  </si>
+  <si>
+    <t>tubba</t>
+  </si>
+  <si>
+    <t>Microtubules</t>
+  </si>
+  <si>
+    <t>CENPA</t>
+  </si>
+  <si>
+    <t>Kinetochore</t>
   </si>
 </sst>
 </file>
@@ -505,7 +550,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7128CD98-9A0B-0D46-9F23-B9C08D30033B}">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
@@ -609,10 +654,88 @@
       <c r="A10" t="s">
         <v>24</v>
       </c>
+      <c r="B10" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>25</v>
+      </c>
+      <c r="B11" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>31</v>
+      </c>
+      <c r="B14" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>33</v>
+      </c>
+      <c r="B15" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>34</v>
+      </c>
+      <c r="B16" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>37</v>
+      </c>
+      <c r="B18" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>38</v>
+      </c>
+      <c r="B19" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>40</v>
+      </c>
+      <c r="B20" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
v11: canonical constructs, marker rollups, and fish seeder
</commit_message>
<xml_diff>
--- a/seed_kits/2025-11-15-121231-autoload/tags.xlsx
+++ b/seed_kits/2025-11-15-121231-autoload/tags.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/davekokel/Projects/carp_v2/seed_kits/2025-11-15-121231-autoload/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C148F9E-36CA-0A4B-B02E-D16F074DACE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1F86C1C-E6BB-584E-8470-BCFB7C3E40E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="34560" windowHeight="19860" xr2:uid="{89706445-C364-CF42-9B42-6F31A2F723ED}"/>
   </bookViews>
@@ -92,9 +92,6 @@
     <t>https://pmc.ncbi.nlm.nih.gov/articles/PMC8716472/</t>
   </si>
   <si>
-    <t>cell cycle</t>
-  </si>
-  <si>
     <t>ER</t>
   </si>
   <si>
@@ -131,9 +128,6 @@
     <t>EB3</t>
   </si>
   <si>
-    <t>Microtubule EBP</t>
-  </si>
-  <si>
     <t>cortactin</t>
   </si>
   <si>
@@ -149,9 +143,6 @@
     <t>LEMD2</t>
   </si>
   <si>
-    <t>Nuclear Envelope</t>
-  </si>
-  <si>
     <t>pex3</t>
   </si>
   <si>
@@ -165,6 +156,15 @@
   </si>
   <si>
     <t>Kinetochore</t>
+  </si>
+  <si>
+    <t>cell_cycle</t>
+  </si>
+  <si>
+    <t>Microtubule_EBP</t>
+  </si>
+  <si>
+    <t>Nuclear_Envelope</t>
   </si>
 </sst>
 </file>
@@ -571,7 +571,7 @@
         <v>15</v>
       </c>
       <c r="E1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
@@ -598,7 +598,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>14</v>
@@ -612,7 +612,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
@@ -620,7 +620,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
@@ -628,10 +628,10 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" t="s">
         <v>20</v>
-      </c>
-      <c r="D7" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
@@ -639,7 +639,7 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
@@ -647,95 +647,95 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B10" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B11" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" t="s">
         <v>27</v>
-      </c>
-      <c r="B12" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B13" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B14" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B15" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B16" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B17" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B18" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B19" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B20" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix tag bug fibrillarilin
</commit_message>
<xml_diff>
--- a/seed_kits/2025-11-15-121231-autoload/tags.xlsx
+++ b/seed_kits/2025-11-15-121231-autoload/tags.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11130"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/davekokel/Projects/carp_v2/seed_kits/2025-11-15-121231-autoload/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1F86C1C-E6BB-584E-8470-BCFB7C3E40E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20E66905-6F65-6C4B-B421-51100002A31D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="34560" windowHeight="19860" xr2:uid="{89706445-C364-CF42-9B42-6F31A2F723ED}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="50">
   <si>
     <t>2Xcox8A</t>
   </si>
@@ -165,13 +165,37 @@
   </si>
   <si>
     <t>Nuclear_Envelope</t>
+  </si>
+  <si>
+    <t>Fibrillarin</t>
+  </si>
+  <si>
+    <t>Nucleolus</t>
+  </si>
+  <si>
+    <t>centrin2</t>
+  </si>
+  <si>
+    <t>Centrioles</t>
+  </si>
+  <si>
+    <t>moesin</t>
+  </si>
+  <si>
+    <t>myosin1A</t>
+  </si>
+  <si>
+    <t>Factin</t>
+  </si>
+  <si>
+    <t>Microvilli</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -190,6 +214,12 @@
       <color rgb="FF1B1B1B"/>
       <name val="Cambria"/>
       <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -212,10 +242,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -550,7 +581,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7128CD98-9A0B-0D46-9F23-B9C08D30033B}">
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
@@ -738,6 +769,38 @@
         <v>38</v>
       </c>
     </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>42</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>44</v>
+      </c>
+      <c r="B22" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>46</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>47</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Rebuild pipeline: apply treatment overrides; update tags seed
</commit_message>
<xml_diff>
--- a/seed_kits/2025-11-15-121231-autoload/tags.xlsx
+++ b/seed_kits/2025-11-15-121231-autoload/tags.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/davekokel/Projects/carp_v2/seed_kits/2025-11-15-121231-autoload/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20E66905-6F65-6C4B-B421-51100002A31D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18D38A72-E454-2442-BDCA-29FA70CCD490}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="34560" windowHeight="19860" xr2:uid="{89706445-C364-CF42-9B42-6F31A2F723ED}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="50">
   <si>
     <t>2Xcox8A</t>
   </si>
@@ -581,7 +581,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7128CD98-9A0B-0D46-9F23-B9C08D30033B}">
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
@@ -801,6 +801,14 @@
         <v>49</v>
       </c>
     </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>28</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>38</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>